<commit_message>
feat: rework certificate portal with phone login and gated articles download
- lookup participants by phone number only and drop the national id column
- add a single sign-in form followed by a menu with certificate and
  proceedings options
- serve articles.zip through download-articles.php for signed-in users
- block direct access to zip and spreadsheet files via .htaccess
</commit_message>
<xml_diff>
--- a/cert/participants.xlsx
+++ b/cert/participants.xlsx
@@ -471,38 +471,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="65" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>کد ملی</t>
+          <t>شماره تماس</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>شماره تماس</t>
+          <t>نام و نام خانوادگی</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>نام و نام خانوادگی</t>
+          <t>عنوان مقاله</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>عنوان مقاله</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>کد گواهی</t>
         </is>
@@ -511,25 +505,20 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>0012345678</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
           <t>09123456789</t>
         </is>
       </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>دکتر سارا محمدی</t>
+        </is>
+      </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>دکتر سارا محمدی</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
           <t>کاربرد هوش مصنوعی مولد در طراحی مراحل بازی‌های نقش‌آفرینی</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>ICCG-2026-101</t>
         </is>
@@ -538,25 +527,20 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>0023456789</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
           <t>09121112233</t>
         </is>
       </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>مهندس علی کریمی</t>
+        </is>
+      </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>مهندس علی کریمی</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
           <t>بهینه‌سازی رندرینگ بلادرنگ در موتورهای بازی‌سازی موبایل</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>ICCG-2026-102</t>
         </is>
@@ -565,25 +549,20 @@
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>0034567890</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
           <t>09351234567</t>
         </is>
       </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>مهدی رضایی</t>
+        </is>
+      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>مهدی رضایی</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
           <t>بررسی روانشناختی تاثیر بازی‌های واقعیت مجازی بر یادگیری تعاملی</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>ICCG-2026-103</t>
         </is>
@@ -592,25 +571,20 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>0045678901</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
           <t>09198765432</t>
         </is>
       </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>زهرا حسینی</t>
+        </is>
+      </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>زهرا حسینی</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
           <t>معماری سرورهای توزیع‌شده برای بازی‌های آنلاین کلان‌مقیاس (MMOG)</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>ICCG-2026-104</t>
         </is>
@@ -619,25 +593,20 @@
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>1234567890</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
           <t>09100000000</t>
         </is>
       </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>پروفسور سید محمدحسین طباطبایی بزرگ‌نیا و همکاران پژوهشی آزمایشگاه ملی بازی‌های رایانه‌ای</t>
+        </is>
+      </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>پروفسور سید محمدحسین طباطبایی بزرگ‌نیا و همکاران پژوهشی آزمایشگاه ملی بازی‌های رایانه‌ای</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
           <t>طراحی، پیاده‌سازی و ارزیابی جامع یک چارچوب مبتنی بر یادگیری تقویتی عمیق و شبکه‌های مولد تخاصمی جهت تولید خودکار و پویا در محیط‌های سه‌بعدی بازی‌های ویدیویی کلان‌مقیاس ابری با تاخیر بسیار پایین</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>ICCG-2026-105</t>
         </is>

</xml_diff>